<commit_message>
corrected the excel errors
</commit_message>
<xml_diff>
--- a/content/english/english-p7-question-bank.xlsx
+++ b/content/english/english-p7-question-bank.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14470" uniqueCount="5384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14470" uniqueCount="5398">
   <si>
     <t>Q_ID</t>
   </si>
@@ -16178,6 +16178,48 @@
   </si>
   <si>
     <t>Manner (gracefully), Place (on the stage), Time (last night).</t>
+  </si>
+  <si>
+    <t>q_id</t>
+  </si>
+  <si>
+    <t>term</t>
+  </si>
+  <si>
+    <t>topic</t>
+  </si>
+  <si>
+    <t>difficulty</t>
+  </si>
+  <si>
+    <t>question_type</t>
+  </si>
+  <si>
+    <t>question_text</t>
+  </si>
+  <si>
+    <t>option_a</t>
+  </si>
+  <si>
+    <t>option_b</t>
+  </si>
+  <si>
+    <t>option_c</t>
+  </si>
+  <si>
+    <t>option_d</t>
+  </si>
+  <si>
+    <t>correct_answer</t>
+  </si>
+  <si>
+    <t>detailed_solution</t>
+  </si>
+  <si>
+    <t>tags</t>
+  </si>
+  <si>
+    <t>hint</t>
   </si>
 </sst>
 </file>
@@ -16200,12 +16242,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -16220,10 +16268,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16507,7 +16556,8 @@
   <dimension ref="A1:O234"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="29.140625" customWidth="1"/>
     <col min="4" max="4" width="40.85546875" customWidth="1"/>
     <col min="5" max="5" width="35.7109375" customWidth="1"/>
@@ -16519,51 +16569,51 @@
     <col min="15" max="15" width="98.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>5384</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5385</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>5386</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>1379</v>
+      <c r="E1" s="3" t="s">
+        <v>5387</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5388</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5389</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>5390</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>5391</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>5392</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>5393</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>5394</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>5395</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>5396</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>5397</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -27527,57 +27577,65 @@
   <dimension ref="A1:BC700"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="89.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.42578125" customWidth="1"/>
+    <col min="9" max="9" width="23.5703125" customWidth="1"/>
+    <col min="10" max="10" width="39.85546875" customWidth="1"/>
+    <col min="11" max="11" width="43.5703125" customWidth="1"/>
+    <col min="12" max="12" width="54.28515625" customWidth="1"/>
+    <col min="13" max="13" width="41.5703125" customWidth="1"/>
+    <col min="14" max="14" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>5384</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5385</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>5386</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>1379</v>
-      </c>
-      <c r="P1" s="2"/>
+      <c r="E1" s="3" t="s">
+        <v>5387</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5388</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5389</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>5390</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>5391</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>5392</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>5393</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>5394</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>5395</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>5396</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>5397</v>
+      </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">

</xml_diff>